<commit_message>
docs: add instruments and care-protocol candidate tables
- 측정도구 시트: 척도 13편 → instrument 13 + S3 공백 1 (문항·응답 척도·시간틀·채점·한국어판·라이선스)
- 프로토콜 시트: 활동 노드 21개(단일 14 · 검증된 다중매체 3 · 실험적 3 · 단계 모듈 1), (프로토콜 × 지표) 등급
- 근거 arm 시트: 프로토콜별 실험 단위 근거 65건(BE experiment_id 후보)
- 등급 규칙·용어(활동 노드 / 중재 / 콘텐츠) 정의, README 갱신

Closes #25

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_측정도구_프로토콜_2026-10-23.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_측정도구_프로토콜_2026-10-23.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BE의 instruments 테이블(측정 노드)과 care_protocols 테이블(중재 노드) 초안. LLM이 생성하지 않고 사람이 검수해 넣는 값</t>
+          <t>BE의 instruments 테이블(측정 노드)과 care_protocols 테이블(활동 노드) 초안. LLM이 생성하지 않고 사람이 검수해 넣는 값</t>
         </is>
       </c>
     </row>
@@ -507,77 +507,89 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>[사전 측정: 공통 앵커 1문항 + 목표별 단축 척도] → [중재 노드 1개] → [사후 측정: 같은 도구] → replan(라운드 2–3회, 중간은 단일 문항만)</t>
+          <t>[사전 측정: 공통 앵커 1문항 + 목표별 단축 척도] → [활동 노드 1개] → [사후 측정: 같은 도구] → replan(라운드 2–3회, 중간은 단일 문항만)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>등급</t>
+          <t>용어</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>'등급 규칙' 시트. (프로토콜 × 결과지표) 쌍 단위로 A/B/C/D, 미측정은 '—'. 상충 근거는 괄호에 논문 ID</t>
+          <t>활동 노드 = 설계·BE 층(Care Protocol 1개 실행, LangGraph run_session). 중재 = 근거·논문 층(근거 arm 시트의 '중재(자극·시간)'). 콘텐츠 = 활동이 쓰는 재료(자연 사진·영상·자연음·안내 음성·도안), prepare가 준비</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>확인 수준</t>
+          <t>등급</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>본문: PDF 본문에서 확인 / 초록: 초록·요약 기준 / 2차: 원문 미확보라 2차 자료·엑셀 기준. 2차 항목은 원문 확보 후 재확인</t>
+          <t>'등급 규칙' 시트. (프로토콜 × 결과지표) 쌍 단위로 A/B/C/D, 미측정은 '—'. 상충 근거는 괄호에 논문 ID</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>원문 미확보</t>
+          <t>확인 수준</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>E02, E13, N06, N10, N23, P30 (6편) / 이미지 PDF(본문 텍스트 없음): N02, N03, N09, P05, P26, P27</t>
+          <t>본문: PDF 본문에서 확인 / 초록: 초록·요약 기준 / 2차: 원문 미확보라 2차 자료·엑셀 기준. 2차 항목은 원문 확보 후 재확인</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BE 반영</t>
+          <t>원문 미확보</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Medium enum에 MUSIC·GUIDED_IMAGERY·WRITING·GROUNDING·ART_VIEWING 추가 필요. Outcome enum의 SUBJECTIVE_STRESS는 상태 불안을 포함하는 것으로 해석</t>
+          <t>E02, E13, N06, N10, N23, P30 (6편) / 이미지 PDF(본문 텍스트 없음): N02, N03, N09, P05, P26, P27</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>S3 공백</t>
+          <t>BE 반영</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>주의·피로의 순간 자가보고 도구가 13편 안에 없음. 과제(SART·BDS)는 세션에 못 넣으므로 VAS 1문항(미검증)으로 두고 외부 도구를 찾아야 함</t>
+          <t>Medium enum에 MUSIC·GUIDED_IMAGERY·WRITING·GROUNDING·ART_VIEWING 추가 필요. Outcome enum의 SUBJECTIVE_STRESS는 상태 불안을 포함하는 것으로 해석</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>S3 공백</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>주의·피로의 순간 자가보고 도구가 13편 안에 없음. 과제(SART·BDS)는 세션에 못 넣으므로 VAS 1문항(미검증)으로 두고 외부 도구를 찾아야 함</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>수집 후보</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>P38 서론이 인용한 Lymeus et al. 2017(실내에서 자연 이미지를 보며 15분 명상)은 S1 핵심 조합(이미지+마음챙김)의 유일한 직접 근거 후보이나 82편 밖</t>
         </is>
@@ -2183,14 +2195,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Care Protocol 후보 — 중재 노드 21개 (단일 14 + 검증된 다중매체 3 + 실험적 3 + 단계 모듈 1)</t>
+          <t>Care Protocol 후보 — 활동 노드 21개 (단일 14 + 검증된 다중매체 3 + 실험적 3 + 단계 모듈 1)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>등급은 (프로토콜 × 결과지표) 쌍 단위('등급 규칙' 시트). 중재 노드는 라운드당 1개, 병행은 '병행 가능' 열의 검증된 조합만. 모든 프로토콜은 MEASURE로 시작·종료하고, 사후 측정은 사전과 같은 도구를 쓴다. PR-13은 E19를 PR-11에 합쳐 결번.</t>
+          <t>등급은 (프로토콜 × 결과지표) 쌍 단위('등급 규칙' 시트). 활동 노드는 라운드당 1개, 병행은 '병행 가능' 열의 검증된 조합만. 모든 프로토콜은 MEASURE로 시작·종료하고, 사후 측정은 사전과 같은 도구를 쓴다. PR-13은 E19를 PR-11에 합쳐 결번.</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2244,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>중재 시간</t>
+          <t>활동 시간</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -2339,7 +2351,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(자연 사진 슬라이드) → NOTICE(선택) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(자연 사진 슬라이드) → NOTICE(선택) → MEASURE</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -2451,7 +2463,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(영상 10분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(영상 10분) → MEASURE</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2563,7 +2575,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(자연 장면) → [사용자 스트레스 상황] → MEASURE</t>
+          <t>MEASURE → ACTIVITY(자연 장면) → [사용자 스트레스 상황] → MEASURE</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -2675,7 +2687,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(자연음) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(자연음) → MEASURE</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -2787,7 +2799,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(음악) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(음악) → MEASURE</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -2899,7 +2911,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(안내 호흡 5분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(안내 호흡 5분) → MEASURE</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -3011,7 +3023,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(녹음 안내 PMR 20분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(녹음 안내 PMR 20분) → MEASURE</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -3119,7 +3131,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(녹음 안내 심상 20분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(녹음 안내 심상 20분) → MEASURE</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -3231,7 +3243,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(오디오 안내 3분) → NOTICE(현재 감각) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(오디오 안내 3분) → NOTICE(현재 감각) → MEASURE</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -3343,7 +3355,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(야외 개방형 명상 20분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(야외 개방형 명상 20분) → MEASURE</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -3455,7 +3467,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(자연 보행) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(자연 보행) → MEASURE</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -3567,7 +3579,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(30분 보행, 좋은 것 3가지 기록) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(30분 보행, 좋은 것 3가지 기록) → MEASURE</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -3679,7 +3691,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(컬러링 20분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(컬러링 20분) → MEASURE</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -3791,7 +3803,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(자연 도안 컬러링 3–5분) → NOTICE → MEASURE</t>
+          <t>MEASURE → ACTIVITY(자연 도안 컬러링 3–5분) → NOTICE → MEASURE</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -4015,7 +4027,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(오감 순서로 알아차리기) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(오감 순서로 알아차리기) → MEASURE</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -4123,7 +4135,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(글쓰기 20분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(글쓰기 20분) → MEASURE</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -4235,7 +4247,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>매일: MEASURE(선택) → INTERVENE(기록 5–10분) → 주 1회 MEASURE</t>
+          <t>매일: MEASURE(선택) → ACTIVITY(기록 5–10분) → 주 1회 MEASURE</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -4347,7 +4359,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(작품 감상 1–2분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(작품 감상 1–2분) → MEASURE</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -4459,7 +4471,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(이미지 보며 명상 15분) → NOTICE → MEASURE</t>
+          <t>MEASURE → ACTIVITY(이미지 보며 명상 15분) → NOTICE → MEASURE</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -4571,7 +4583,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>MEASURE → INTERVENE(이미지 + 안내 호흡 5분) → MEASURE</t>
+          <t>MEASURE → ACTIVITY(이미지 + 안내 호흡 5분) → MEASURE</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -8894,7 +8906,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>중재 노드 라운드당 1개. 순차는 라운드 사이(replan)에서만, 사이에 MEASURE 필수. 라운드 2–3회 제한, 중간 측정은 단일 문항(INS-SAM/INS-GRID)</t>
+          <t>활동 노드 라운드당 1개. 순차는 라운드 사이(replan)에서만, 사이에 MEASURE 필수. 라운드 2–3회 제한, 중간 측정은 단일 문항(INS-SAM/INS-GRID)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: add N27 mental fatigue instrument review and replace INS-GAP-S3 with INS-MFVAS
- 00_original_PDF: N27 Díaz-García et al. (2022) 원문 추가 — PMC8744873 OA 출판본, CC BY, 텍스트층 있음
- 논문목록: N27을 R1·R5 블록 끝에 등재(RAG별 연결 196건), 논문 유형 기준 체계적 고찰 18편·합계 83편
- 측정도구·프로토콜 워크북: 측정도구 시트 INS-GAP-S3 행을 INS-MFVAS(정신 피로 VAS 3문항, 미검증, 출처 N27)로 갱신하고 프로토콜·요약·등급 규칙 시트의 참조를 맞춤
- README: N27 추가 경위, 현재 상태 83편 / 77편 / 6편

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_측정도구_프로토콜_2026-10-23.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_측정도구_프로토콜_2026-10-23.xlsx
@@ -463,6 +463,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -471,7 +472,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-23 · 2026-10-27 S3 임시 도구(INS-MFVAS) 반영</t>
         </is>
       </c>
     </row>
@@ -483,7 +484,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>LUMI_R_C_논문목록_2026-10-22.xlsx 82편 — 척도·측정도구 13편 → '측정도구', 무작위 실험 35편 + 준실험 7편 → '프로토콜'·'근거 arm'</t>
+          <t>LUMI_R_C_논문목록_2026-10-22.xlsx 83편 — 척도·측정도구 13편(+ S3 VAS 형식 근거 체계적 고찰 N27) → '측정도구', 무작위 실험 35편 + 준실험 7편 → '프로토콜'·'근거 arm'</t>
         </is>
       </c>
     </row>
@@ -574,12 +575,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>S3 공백</t>
+          <t>S3 임시 도구</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>주의·피로의 순간 자가보고 도구가 13편 안에 없음. 과제(SART·BDS)는 세션에 못 넣으므로 VAS 1문항(미검증)으로 두고 외부 도구를 찾아야 함</t>
+          <t>주의·피로의 순간 자가보고 검증 도구가 13편 안에 없음. 과제(SART·BDS)는 세션에 못 넣으므로 팀이 쓴 정신 피로 VAS 3문항(INS-MFVAS, 미검증·BE status PROVISIONAL)으로 주관적 피로만 재고 판정은 fatigue↓. VAS 형식의 근거는 N27(정신 피로·부하 측정 도구 체계적 고찰)이고 문항 자체는 검증되지 않았으므로 검증 도구 탐색은 계속. 측정 지표(주관적 피로)가 근거의 S3 1차 지표(과제로 잰 주의)와 다르다는 것을 Reference 카드에 표시</t>
         </is>
       </c>
     </row>
@@ -637,7 +638,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>측정도구 (instruments) — 척도·측정도구 13편 + S3 공백 1건</t>
+          <t>측정도구 (instruments) — 척도·측정도구 13편 + S3 임시 도구 1건(INS-MFVAS)</t>
         </is>
       </c>
     </row>
@@ -648,6 +649,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -1651,22 +1653,22 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>INS-GAP-S3</t>
+          <t>INS-MFVAS</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>(공백) 순간 피로·주의 자가보고</t>
+          <t>정신 피로 VAS (Mental Fatigue VAS) — 임시 도구</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N27</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LUMI 팀 문항(2026-10-27) · 형식 근거 Díaz-García et al. 2022</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1676,17 +1678,17 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>순간 정신 피로 / 주관적 주의 집중</t>
+          <t>순간 정신 피로(주관) — 피로감 · 집중 어려움 · 기운</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>1 (제안: VAS)</t>
+          <t>3 (fatigue 피로 · concentration 집중 어려움 · energy 기운)</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>0–100 VAS(제안)</t>
+          <t>0–100 슬라이더(1단위), 문항별 양끝 라벨(예: 전혀 피로하지 않다 – 매우 피로하다)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1696,17 +1698,17 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>단일 값</t>
+          <t>문항별 0–100 그대로(합산 없음). energy는 높을수록 좋음</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>미검증</t>
+          <t>미검증. 절단점 없음(변화량). 개선 판정은 fatigue 1문항 감소(fatigue↓)만 쓰고 concentration·energy는 수집용</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— (미검증)</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -1716,7 +1718,7 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>S3 사전·사후 임시 도구. '미검증' 표시 필수. 외부 도구 탐색 과제</t>
+          <t>S3 목표 척도이자 라운드 척도 — 사전·라운드마다 SAM과 함께 재고 종료 때 다시 묻지 않음(마지막 사후값 = 종료값). '미검증' 표시 필수</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -1726,27 +1728,27 @@
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>팀이 한국어로 쓴 문항(번역 아님)</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>팀 작성 문항 — 외부 사용 허가 불필요</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>확보(텍스트)</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>본문</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>13편 내 순간 피로·주의 자가보고 도구 없음. 근거 실험은 과제(SART·BDS·LDST)로 측정</t>
+          <t>BE data/instruments/INS-MFVAS.json(status PROVISIONAL, BE PR #37). N27은 서론의 '정신 피로는 VAS가 가장 많이 쓰인 도구' 서술(인용 없음)로 VAS 형식의 근거일 뿐 3문항을 검증하지 않음. N27이 정리한 검증 도구는 대부분 기간 시간틀 다문항 척도(CFQ·MFI 등)이고, 표 2의 STI-CF(상태·특성판, 65세 이상 표본)는 교체 후보 — 원문 확인 필요. concentration 문항은 N03 정신 피로 하위척도 문항을 '지금' 시간틀로 옮김. 주의 용량은 재지 않음 — 근거 실험의 S3 지표(과제 SART·BDS·LDST)와 다름. 사용자 데이터로 문항 간 상관·신뢰도를 본 뒤 유지·교체 결정</t>
         </is>
       </c>
     </row>
@@ -2206,6 +2208,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -2411,7 +2414,7 @@
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>INS-SAM(앵커) + S2: INS-STAI6 / S3: INS-GAP-S3</t>
+          <t>INS-SAM(앵커) + S2: INS-STAI6 / S3: INS-MFVAS</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
@@ -2747,7 +2750,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>INS-SAM(앵커) + S3: INS-GAP-S3</t>
+          <t>INS-SAM(앵커) + S3: INS-MFVAS</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -3415,7 +3418,7 @@
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t>INS-SAM(앵커) + INS-GAP-S3</t>
+          <t>INS-SAM(앵커) + INS-MFVAS</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
@@ -3527,7 +3530,7 @@
       </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
-          <t>INS-SAM(앵커) + INS-GAP-S3</t>
+          <t>INS-SAM(앵커) + INS-MFVAS</t>
         </is>
       </c>
       <c r="T15" s="3" t="inlineStr">
@@ -4708,6 +4711,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -8698,6 +8702,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -8906,7 +8911,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>활동 노드 라운드당 1개. 순차는 라운드 사이(replan)에서만, 사이에 MEASURE 필수. 라운드 2–3회 제한, 중간 측정은 단일 문항(INS-SAM/INS-GRID)</t>
+          <t>활동 노드 라운드당 1개. 순차는 라운드 사이(replan)에서만, 사이에 MEASURE 필수. 라운드 2–3회 제한, 중간 측정은 단일 문항(INS-SAM/INS-GRID). 예외: S3는 INS-MFVAS(슬라이더 3개)를 사전·라운드마다 함께 재고 종료 때 다시 묻지 않음</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: register BSRI original paper N28 and rename the author overview PDF
- 00_original_PDF: BSRI 저자 척도 소개 문서(문항 · 채점 · 사용 조건)를 N28_2018_Marchetti_BSRI_author_overview_items_and_scoring.pdf로 이름 변경 — 2018 논문 원문이 아니다
- LUMI_R_C_논문목록: N28(Marchetti 외 2018) R1 · R2 · R5 행 추가, 논문 유형 기준 척도 14편 · 합계 84편 (BE manifest와 맞춤)
- 미확보_논문_직접검색_목록: N28 추가(총 7편)
- LUMI_측정도구_프로토콜: INS-BSRI 출처 N28 · 원판 연도 2014 → 2018 · 채점(저자 합계 0–800, LUMI 평균) · 한국어판(번역 초안) · 라이선스(연구 목적 무료) · 원문 확보, INS-STAI6 한국어판, 요약 시트
- README: N28과 척도 소개 문서, 현재 상태 84 · 77 · 7

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_R_C_Research_2026-10-22/LUMI_측정도구_프로토콜_2026-10-23.xlsx
+++ b/LUMI_R_C_Research_2026-10-22/LUMI_측정도구_프로토콜_2026-10-23.xlsx
@@ -463,7 +463,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -472,7 +471,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23 · 2026-10-27 S3 임시 도구(INS-MFVAS) 반영</t>
+          <t>2026-10-23 · 2026-10-27 S3 임시 도구(INS-MFVAS) 반영 · 2026-10-29 BSRI 원판 N28 등재(원문 미확보, 저자 척도 소개 문서 확보) · STAI-6·BSRI 번역 초안(BE #79) 반영</t>
         </is>
       </c>
     </row>
@@ -484,7 +483,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>LUMI_R_C_논문목록_2026-10-22.xlsx 83편 — 척도·측정도구 13편(+ S3 VAS 형식 근거 체계적 고찰 N27) → '측정도구', 무작위 실험 35편 + 준실험 7편 → '프로토콜'·'근거 arm'</t>
+          <t>LUMI_R_C_논문목록_2026-10-22.xlsx 84편 — 척도·측정도구 14편(+ S3 VAS 형식 근거 체계적 고찰 N27) → '측정도구', 무작위 실험 35편 + 준실험 7편 → '프로토콜'·'근거 arm'</t>
         </is>
       </c>
     </row>
@@ -556,7 +555,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>E02, E13, N06, N10, N23, P30 (6편) / 이미지 PDF(본문 텍스트 없음): N02, N03, N09, P05, P26, P27</t>
+          <t>E02, E13, N06, N10, N23, N28, P30 (7편) / 이미지 PDF(본문 텍스트 없음): N02, N03, N09, P05, P26, P27</t>
         </is>
       </c>
     </row>
@@ -649,7 +648,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -1034,7 +1032,7 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>STAI 전체판 한국어 타당화 연구 있음(확인 필요). 6문항 단축형 한국어 검증은 확인 필요</t>
+          <t>STAI 전체판 한국어 타당화 연구 있음(확인 필요). 6문항 단축형 한국어 검증은 확인 필요 → LUMI 내부 시험용 번역 초안(PROVISIONAL, BE #79)</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -1067,12 +1065,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>N25</t>
+          <t>N28 · N25</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Marchetti et al. 2014; Chiorri et al. 2026</t>
+          <t>Marchetti et al. 2018; Chiorri et al. 2026</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1102,7 +1100,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>합 0–800 또는 평균</t>
+          <t>8문항 합 0–800(저자 기준, 모두 정방향). LUMI는 평균(합 ÷ 8, 0–100)</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1112,7 +1110,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>이탈리아 성인(지필 N=216, 온라인 N=222, N=675); 영어 원판 Marchetti 2014</t>
+          <t>이탈리아 성인(지필 N=216, 온라인 N=222, N=675); 영어 원판 Marchetti 2018</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1132,17 +1130,17 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>미확인 → 번역·타당화 필요(LLM 번역 금지)</t>
+          <t>검증된 한국어판 없음(저자 소개 문서: 한국어 번역은 있으나 미검증) → LUMI 내부 시험용 번역 초안(PROVISIONAL, BE #79)</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>논문 게재, 무료(확인)</t>
+          <t>연구 목적 무료 사용 — Marchetti et al. 2018 인용(저자 척도 소개 문서)</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>확보(텍스트)</t>
+          <t>N25 확보(텍스트) · N28 원문 미확보 — 저자 척도 소개 문서 확보</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
@@ -2208,7 +2206,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -4711,7 +4708,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -8702,7 +8698,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>

</xml_diff>